<commit_message>
Add synthetic batch numbers and product group counts, state authorship as evidenced
- Synthetic cases get a Batch column (SYN-LOT-<year><letter><number>); two cases share batch SYN-LOT-26A019.
- Statistics, prompt and report add counts by product group and a list of batches with more than one case; the case list shows product group and batch.
- Prewritten demo answer updated to the new statistics; it cites only existing case IDs.
- README "My role": requirements and scope by Nikita; code, tests and docs written by an AI coding agent.
- Design note: "trained QA reviewer" instead of "qualified person", neutral voice in the risk view, GAMP 5 Second Edition (2022) Appendix D11 cited with title.
- Prompt: "trained QA reviewer"; batch numbers are written without brackets so the case ID check does not flag them.
- docs/sample regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/cases.xlsx
+++ b/samples/cases.xlsx
@@ -55,8 +55,10 @@
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="90" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="90" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -89,15 +91,20 @@
       </c>
       <c r="E2" t="inlineStr" s="2">
         <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr" s="2">
+        <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr" s="2">
+      <c r="G2" t="inlineStr" s="2">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr" s="2">
+      <c r="H2" t="inlineStr" s="2">
         <is>
           <t>Description</t>
         </is>
@@ -124,15 +131,20 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-25A112</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t xml:space="preserve">Closed</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t xml:space="preserve">Outer carton dented on one corner. Blister intact, no tablets missing.</t>
         </is>
@@ -159,15 +171,20 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-25B041</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t xml:space="preserve">Major</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t xml:space="preserve">Closed</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t xml:space="preserve">Expiry date on the bottle label partly illegible. Carton print is readable.</t>
         </is>
@@ -194,15 +211,20 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26A003</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t xml:space="preserve">Closed</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t xml:space="preserve">Two tablets in one blister show small dark specks on the surface.</t>
         </is>
@@ -229,15 +251,20 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-25C077</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t xml:space="preserve">Closed</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t xml:space="preserve">Blister foil torn at one cavity on arrival. Capsule present and intact.</t>
         </is>
@@ -264,15 +291,20 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26B006</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Major</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t xml:space="preserve">Open</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t xml:space="preserve">Measuring cup missing from the carton.</t>
         </is>
@@ -299,15 +331,20 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26A011</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t xml:space="preserve">Open</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t xml:space="preserve">Carton crushed in transport. The shipping box was also damaged.</t>
         </is>
@@ -334,15 +371,20 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26D002</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t xml:space="preserve">Critical</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t xml:space="preserve">Open</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t xml:space="preserve">Customer reports a dark fibre in the cream after first opening of the tube. Sample requested.</t>
         </is>
@@ -369,15 +411,20 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26C009</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t xml:space="preserve">Open</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t xml:space="preserve">Two cartons in one shipment dented. Contents not affected.</t>
         </is>
@@ -404,15 +451,20 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26A019</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t xml:space="preserve">Open</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t xml:space="preserve">Patient leaflet missing from the carton.</t>
         </is>
@@ -439,15 +491,20 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26A019</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Major</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t xml:space="preserve">Open</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t xml:space="preserve">Blister strip cracked across two cavities, one tablet broken. Customer asked for a call back on +49 30 5550 1234.</t>
         </is>
@@ -470,7 +527,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Case IDs, dates, products and texts are invented. Any resemblance to real complaints is accidental.</t>
+          <t>Case IDs, batch numbers (SYN-LOT-...), dates, products and texts are invented. Any resemblance to real complaints is accidental.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add synthetic batch numbers and product group counts, state authorship as evidenced (#3)
Synthetic SYN-LOT batch numbers and product group counts in statistics, prompt and report; demo answer and docs/sample regenerated (CI run 40996837685); README My role and design note reworded to the evidenced authorship; trained QA reviewer instead of qualified person; GAMP 5 Second Edition (2022) Appendix D11 cited.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/cases.xlsx
+++ b/samples/cases.xlsx
@@ -55,8 +55,10 @@
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="90" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="90" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -89,15 +91,20 @@
       </c>
       <c r="E2" t="inlineStr" s="2">
         <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr" s="2">
+        <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr" s="2">
+      <c r="G2" t="inlineStr" s="2">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr" s="2">
+      <c r="H2" t="inlineStr" s="2">
         <is>
           <t>Description</t>
         </is>
@@ -124,15 +131,20 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-25A112</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t xml:space="preserve">Closed</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t xml:space="preserve">Outer carton dented on one corner. Blister intact, no tablets missing.</t>
         </is>
@@ -159,15 +171,20 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-25B041</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t xml:space="preserve">Major</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t xml:space="preserve">Closed</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t xml:space="preserve">Expiry date on the bottle label partly illegible. Carton print is readable.</t>
         </is>
@@ -194,15 +211,20 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26A003</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t xml:space="preserve">Closed</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t xml:space="preserve">Two tablets in one blister show small dark specks on the surface.</t>
         </is>
@@ -229,15 +251,20 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-25C077</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t xml:space="preserve">Closed</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t xml:space="preserve">Blister foil torn at one cavity on arrival. Capsule present and intact.</t>
         </is>
@@ -264,15 +291,20 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26B006</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Major</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t xml:space="preserve">Open</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t xml:space="preserve">Measuring cup missing from the carton.</t>
         </is>
@@ -299,15 +331,20 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26A011</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t xml:space="preserve">Open</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t xml:space="preserve">Carton crushed in transport. The shipping box was also damaged.</t>
         </is>
@@ -334,15 +371,20 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26D002</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t xml:space="preserve">Critical</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t xml:space="preserve">Open</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t xml:space="preserve">Customer reports a dark fibre in the cream after first opening of the tube. Sample requested.</t>
         </is>
@@ -369,15 +411,20 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26C009</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t xml:space="preserve">Open</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t xml:space="preserve">Two cartons in one shipment dented. Contents not affected.</t>
         </is>
@@ -404,15 +451,20 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26A019</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t xml:space="preserve">Open</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t xml:space="preserve">Patient leaflet missing from the carton.</t>
         </is>
@@ -439,15 +491,20 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t xml:space="preserve">SYN-LOT-26A019</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Major</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t xml:space="preserve">Open</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t xml:space="preserve">Blister strip cracked across two cavities, one tablet broken. Customer asked for a call back on +49 30 5550 1234.</t>
         </is>
@@ -470,7 +527,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Case IDs, dates, products and texts are invented. Any resemblance to real complaints is accidental.</t>
+          <t>Case IDs, batch numbers (SYN-LOT-...), dates, products and texts are invented. Any resemblance to real complaints is accidental.</t>
         </is>
       </c>
     </row>

</xml_diff>